<commit_message>
📅 日报更新 2026-08-30 07:04
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-08-30.xlsx
+++ b/data/exports/黄老师/dist_order_2026-08-30.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49782066</v>
+        <v>49826011</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>前程似锦 </t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49771027</v>
+        <v>49825720</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49673360</v>
+        <v>49825676</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -284,7 +284,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49673352</v>
+        <v>49825650</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -344,7 +344,7 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49673350</v>
+        <v>49825642</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -404,7 +404,7 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49673349</v>
+        <v>49825640</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -464,7 +464,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>49646935</v>
+        <v>49825639</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>49646933</v>
+        <v>49825637</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>49646901</v>
+        <v>49825635</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
@@ -665,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>49646876</v>
+        <v>49825628</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J11" s="0" t="inlineStr">
@@ -725,11 +725,11 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>49646867</v>
+        <v>49782066</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>前程似锦 </t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -785,11 +785,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>49636232</v>
+        <v>49771027</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -845,11 +845,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>49636184</v>
+        <v>49673360</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -905,11 +905,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>49636170</v>
+        <v>49673352</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
@@ -965,11 +965,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>49636157</v>
+        <v>49673350</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="I16" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J16" s="0" t="inlineStr">
@@ -1025,11 +1025,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>49593974</v>
+        <v>49673349</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
@@ -1085,11 +1085,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>49593671</v>
+        <v>49646935</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
@@ -1145,11 +1145,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>49535916</v>
+        <v>49646933</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J19" s="0" t="inlineStr">
@@ -1205,11 +1205,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>49535653</v>
+        <v>49646901</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -1265,11 +1265,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>49535650</v>
+        <v>49646876</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
@@ -1320,21 +1320,16 @@
       <c r="L21" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N21" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>49508265</v>
+        <v>49646867</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1359,7 +1354,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1369,7 +1364,7 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
@@ -1390,11 +1385,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>49493414</v>
+        <v>49636232</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1419,7 +1414,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1450,11 +1445,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>49493126</v>
+        <v>49636184</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1479,7 +1474,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1489,7 +1484,7 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
@@ -1510,11 +1505,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>49492499</v>
+        <v>49636170</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1539,7 +1534,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1549,7 +1544,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J25" s="0" t="inlineStr">
@@ -1570,11 +1565,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>49455301</v>
+        <v>49636157</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1599,7 +1594,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1609,7 +1604,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
@@ -1630,11 +1625,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>49432023</v>
+        <v>49593974</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1659,7 +1654,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1690,11 +1685,11 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>49415939</v>
+        <v>49593671</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1719,7 +1714,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1729,17 +1724,17 @@
       </c>
       <c r="I28" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J28" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K28" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L28" s="0" t="inlineStr">
@@ -1750,11 +1745,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>49415918</v>
+        <v>49535916</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1779,7 +1774,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1789,17 +1784,17 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
@@ -1810,11 +1805,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>49415913</v>
+        <v>49535653</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1839,7 +1834,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1849,17 +1844,17 @@
       </c>
       <c r="I30" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J30" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K30" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L30" s="0" t="inlineStr">
@@ -1870,11 +1865,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>49415890</v>
+        <v>49535650</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1899,7 +1894,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1909,17 +1904,17 @@
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K31" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L31" s="0" t="inlineStr">
@@ -1929,17 +1924,17 @@
       </c>
       <c r="N31" s="0" t="inlineStr">
         <is>
-          <t>宜春</t>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>49415874</v>
+        <v>49508265</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1964,7 +1959,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1974,17 +1969,17 @@
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J32" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K32" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L32" s="0" t="inlineStr">
@@ -1995,11 +1990,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>49415871</v>
+        <v>49493414</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2024,7 +2019,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2034,17 +2029,17 @@
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L33" s="0" t="inlineStr">
@@ -2055,59 +2050,664 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
+        <v>49493126</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>刘盼昭</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G34" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:44:53</t>
+        </is>
+      </c>
+      <c r="H34" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J34" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K34" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L34" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="0">
+        <v>49492499</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>红霞</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F35" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G35" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:29:43</t>
+        </is>
+      </c>
+      <c r="H35" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J35" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K35" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L35" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="0">
+        <v>49455301</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>周开平</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G36" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 22:46:59</t>
+        </is>
+      </c>
+      <c r="H36" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J36" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K36" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L36" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="0">
+        <v>49432023</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>花生米</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E37" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F37" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G37" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:55:45</t>
+        </is>
+      </c>
+      <c r="H37" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J37" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K37" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L37" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="0">
+        <v>49415939</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>杨梅芳</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E38" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G38" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:58</t>
+        </is>
+      </c>
+      <c r="H38" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I38" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J38" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K38" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L38" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="A39" s="0">
+        <v>49415918</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>心语无言</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G39" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:24</t>
+        </is>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J39" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K39" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L39" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G40" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J40" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K40" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L40" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I41" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J41" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K41" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L41" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N41" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
+      <c r="A42" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I42" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J42" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K42" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L42" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
+      <c r="A43" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I43" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J43" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K43" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L43" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="A44" s="0">
         <v>49415867</v>
       </c>
-      <c r="B34" s="0" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C34" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D34" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E34" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F34" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G34" s="0" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G44" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H34" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" s="0" t="inlineStr">
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I44" s="0" t="inlineStr">
         <is>
           <t>黄老师-抖音01</t>
         </is>
       </c>
-      <c r="J34" s="0" t="inlineStr">
+      <c r="J44" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K34" s="0" t="inlineStr">
+      <c r="K44" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L34" s="0" t="inlineStr">
+      <c r="L44" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>